<commit_message>
📊 Horarios actualizados Línea 141 - 5053
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-09.xlsx
+++ b/data/horarios-141-2026-10-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:05</t>
+          <t>Última actualización: 12:13:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -733,7 +733,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1015,6 +1015,856 @@
         <v>117</v>
       </c>
       <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>12:16</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>12:17</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:18</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>83_ESC 6_ALUAR</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>8</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>12:24</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>17_179 Y 38</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>11</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>12</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>12</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>19</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>20</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>20</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>12:39</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>26</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>27</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>32</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>12:48</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>35</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>36</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>37</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>44</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>47</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>57</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>13:12</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>59</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>68</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>72</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>72</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>76</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>13:36</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>83</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>100</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>101</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>104</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>107</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>14:05</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>112</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>113</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1031,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1044,14 +1894,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:05</t>
+          <t>Última actualización: 12:13:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1177,6 +2027,81 @@
         <v>98</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>12</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>72</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>113</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1193,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1206,14 +2131,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:01:05</t>
+          <t>Última actualización: 12:13:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1316,6 +2241,131 @@
       <c r="E8" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>45</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>58</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>62</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>13:27</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_ESC AGRARIA-LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>74</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>12:13:39</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>91</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5054
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-09.xlsx
+++ b/data/horarios-141-2026-10-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:13:39</t>
+          <t>Última actualización: 17:06:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 56</t>
+          <t>Total filas: 88</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -733,7 +733,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1865,6 +1865,806 @@
         <v>113</v>
       </c>
       <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>17:09</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>3</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>4</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>4</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>17:17</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>11</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>17:20</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>14</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>15</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>16</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>17:26</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>20</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>17:31</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>25</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>32</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>34</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>17:40</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>34</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>17:41</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>35</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>17:46</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>40</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>41</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>46</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>17:55</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>49</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>54</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>83_ESC 6_ALUAR</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>59</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>18:09</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>63</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>70</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>78</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>78</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>18:29</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>83</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>84</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>85</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>94</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>95</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>100</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>102</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>109</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>19:04</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>118</v>
+      </c>
+      <c r="E93" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1881,7 +2681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1894,14 +2694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:13:39</t>
+          <t>Última actualización: 17:06:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2102,6 +2902,106 @@
         <v>113</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>95</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>100</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>102</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2118,7 +3018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2131,14 +3031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:13:39</t>
+          <t>Última actualización: 17:06:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -2364,6 +3264,131 @@
         <v>91</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>17:14</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>17:27</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>21</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>18:41</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>103</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>17:06:58</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>108</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 5055
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-10-09.xlsx
+++ b/data/horarios-141-2026-10-09.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:06:58</t>
+          <t>Última actualización: 20:58:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 88</t>
+          <t>Total filas: 105</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -733,7 +733,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1333,7 +1333,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D63" t="n">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>26_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>26_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2665,6 +2665,431 @@
         <v>118</v>
       </c>
       <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>21:05</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>7</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>21:12</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>14</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>21:18</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>20</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>21:19</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>21</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>21:20</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>22</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>28</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>32</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>34</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>21:35</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>37</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>48</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>62</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>22:08</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>70</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>22:20</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>82</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>84</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>22:31</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>93</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>22:38</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>100</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>22:57</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>119</v>
+      </c>
+      <c r="E110" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2681,7 +3106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2694,14 +3119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:06:58</t>
+          <t>Última actualización: 20:58:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -3002,6 +3427,31 @@
         <v>102</v>
       </c>
       <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>22:57</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>119</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3018,7 +3468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3031,14 +3481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:06:58</t>
+          <t>Última actualización: 20:58:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3389,6 +3839,106 @@
         <v>108</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>21:07</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>9</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>21:57</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>59</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>74</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>20:58:55</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>22:21</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>83</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>